<commit_message>
Bug fix for the Excel annotations file
</commit_message>
<xml_diff>
--- a/rag/judge-subset/Annotations-flan-t5-large.xlsx
+++ b/rag/judge-subset/Annotations-flan-t5-large.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>where is the lady with an ermine located</t>
+          <t>what is the meaning of lc in banking</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -491,7 +491,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>the National Museum in Kraków</t>
+          <t>letter of credit</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>lok sabha or rajya sabha which is bigger</t>
+          <t>what engines do they use in formula 1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -530,7 +530,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Lok Sabha</t>
+          <t>1.6 litre V6 turbo engines</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>who was the actress who played pinky tuscadero on happy days</t>
+          <t>who is the presiding officer in the house</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Roz Kelly</t>
+          <t>The Speaker of the House</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>who wrote the song i want you back</t>
+          <t>who won the 2002 us open men's tennis championship</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Berry GordyFreddie PerrenAlphonso MizellDeke Richards</t>
+          <t>Pete Sampras</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>who wrote the music for fiddler on the roof</t>
+          <t>who played the original charlie and the chocolate factory</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Jerry Bock</t>
+          <t>Peter Gardner[4] Ostrum</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>who sang last night a dj saved my life</t>
+          <t>number of cities and towns in rhode island</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Réjane "Reggie" MagloireRose Marie Ramsey</t>
+          <t>8 cities31 towns</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>where is the women's world cup being held</t>
+          <t>who won the australian men's open final</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Roger Federer</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>what city does big bang theory take place</t>
+          <t>who played john ross ewing in the original dallas</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Pasadena, California</t>
+          <t>Omri Katz</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>when did the first goosebumps book come out</t>
+          <t>the release of an egg cell is called</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>July 1992</t>
+          <t>ovulation</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ethics comes from the greek word 'ethos' which means</t>
+          <t>who plays dr shepherd on grey's anatomy</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>"character"</t>
+          <t>Patrick Dempsey</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>who said what's done is done in macbeth</t>
+          <t>where did frodo have to take the ring</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Lady Macbeth</t>
+          <t>Mount Doom</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>when did wizard of oz air on tv</t>
+          <t>where is all the raw data processed in a pc</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>November 3, 1956</t>
+          <t>hard disk drives</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>what is the most established and iconic instrumental ensemble in western culture</t>
+          <t>where is a sunday afternoon on the island of la grande jatte located</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>bluegrass</t>
+          <t>the Art Institute of Chicago</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>manchester utd vs manchester city head to head</t>
+          <t>who did the original version of the song signs</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Manchester derby</t>
+          <t>Canadian rock group Five Man Electrical Band</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>where does the young and the restless film</t>
+          <t>what are tiny pores present on the surface of leaf called</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>at CBS Television City, studios 41 and 43 in Hollywood</t>
+          <t>stomates</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>who does the us department of justice report to</t>
+          <t>how much did germany have to pay in ww1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>United States Attorney General</t>
+          <t>132 billion gold marks</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>how many chapters are in the book of proverbs</t>
+          <t>who played aunt esther on sanford and son</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>LaWanda Page</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>when did the only way is essex first start</t>
+          <t>which province of canada has a large french population</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>10 October 2010</t>
+          <t>Quebec</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>which organelle makes the digestive enzymes of lysosome</t>
+          <t>when did papua new guinea become an independent country</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>the Golgi apparatus</t>
+          <t>16 September 1975</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>where is the first in n out burger located</t>
+          <t>when does the school year start in israel</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Baldwin Park, California</t>
+          <t>September 1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>what is the name of agarbatti in english</t>
+          <t>who sang vocals on wish you were here</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>incense sticks</t>
+          <t>David Gilmour</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>who sings the theme song from robin hood prince of thieves</t>
+          <t>when is the movie a wrinkle in time coming out</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Michael Kamen</t>
+          <t>March 9, 2018</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>who painted the woman with the pearl earring</t>
+          <t>unix command to copy a folder from one location to another</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Johannes Vermeer</t>
+          <t>cp</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>who gets to be the speaker of the house</t>
+          <t>who founded the mormon faith in new york</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>presiding officer of the United States House of Representatives</t>
+          <t>Joseph Smith</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>what kind of peppers are in a greek salad</t>
+          <t>who is the mother of moses in the holy bible</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>pickled hot peppersbell peppers</t>
+          <t>Jochebed</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>who wrote come thou fount of every blessing lyrics</t>
+          <t>where is eden west resort from couples retreat</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Robert Robinson</t>
+          <t>Bora Bora</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>when was video killed the radio star released</t>
+          <t>when did pak n save open in nz</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>7 September 1979</t>
+          <t>June 1985</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>what nfl football team has the most superbowl rings</t>
+          <t>tom cruise movie where he dies and comes back to life</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Pittsburgh Steelers</t>
+          <t>Edge of Tomorrow (also known by its marketing tagline Live. Die. Repeat.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>who is the chief judge of allahabad high court</t>
+          <t>what is the altitude of the sacred valley</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Dilip Babasaheb Bhosale</t>
+          <t>ranging from 3,000 metres (9,800 ft) at Pisac to 2,050 metres (6,730 ft)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>where did serena van der woodsen go to college</t>
+          <t>when did they add ain't to the dictionary</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>1961</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>who has held chief minister office for longest period of time</t>
+          <t>who has home field advantage in the alds</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Pawan Kumar Chamling</t>
+          <t>the team with the better regular season record</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>who won the battle of ramsour's mill</t>
+          <t>where is the diamond cutting industry located in india</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Patriot militia</t>
+          <t>Surat</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>when did north korea join the united nations</t>
+          <t>when did the yankees move to new stadium</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>17 September 1991</t>
+          <t>in 2009</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>how many dunk and egg stories are there</t>
+          <t>how many books can i upload to google books</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Three</t>
+          <t>up to 1,000</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>how many countries negotiated the iran nuclear deal</t>
+          <t>when did lego first begin licensing characters from movie and tv shows for lego sets</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>GermanyChinaFranceRussiathe United Kingdomthe United StatesIslamic Republic of IranEuropean Union</t>
+          <t>1999</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>when was the term great britain first used</t>
+          <t>in which language is the indian national anthem</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>1474</t>
+          <t>Bengali</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>who commanded the british attack on quebec quizlet</t>
+          <t>what sports did they do in ancient greece olympics</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>General James Wolfe</t>
+          <t>foot race</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>who joined america after the battle of saratoga</t>
+          <t>manchester utd vs manchester city head to head</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Manchester derby</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>which type of wastewater treatment involves forcing the wastewater through a semipermeable membrane</t>
+          <t>where do they get the tree for rockefeller center</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Reverse osmosis</t>
+          <t>upstate New York and surrounding states, and even Ottawa, Canada</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>who sings you just call out my name</t>
+          <t>who had the first dunk in nba history</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>The Weeknd</t>
+          <t>center and Olympic Gold Medalist Bob Kurland</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>who controls the amount of money in circulation</t>
+          <t>who won the match race between seabiscuit and war admiral</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>central banks such as the United States Federal Reserve System, the European Central Bank (ECB), and the People's Bank of China</t>
+          <t>Seabiscuit</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>average distance from earth to sun in kilometers</t>
+          <t>the name given to the east to west rotation of venus</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>about 150 million</t>
+          <t>retrograde</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>how do they test for weed in your system</t>
+          <t>who gets murdered in the man in 3b</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>urinalysishair analysissaliva tests</t>
+          <t>Darryl</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>who wrote the song don t want to miss a thing</t>
+          <t>when does war of planet of the apes come out</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Diane Warren</t>
+          <t>July 14, 2017</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>who sang take it to the limit for the eagles</t>
+          <t>the first buddhist council was held in the region of</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Randy Meisner</t>
+          <t>Sattapanni caves Rajgriha (now Rajgir)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>where was the first offshore oil well drilled</t>
+          <t>who is the voice on michael jackson thriller</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>in the fresh waters of the Grand Lake St. Marys (a.k.a. Mercer County Reservoir) in Ohio</t>
+          <t>Vincent Price</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>how many oscars did fellowship of the ring win</t>
+          <t>who played jackie in fresh prince of bel air</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>four</t>
+          <t>Tyra Banks</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>who signs the assignment of deed of trust</t>
+          <t>electrical impulses are conducted efficiently through cardia muscle via</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>the borrower/trustor</t>
+          <t>the Purkinje fibers</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>when did lion king come out in theaters</t>
+          <t>which three nations participated in the d-day operations in normandy</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>June 24, 1994</t>
+          <t>the Americansthe Britishthe Canadians</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>what musical is the song there's a place for us</t>
+          <t>a bundle of sticks that starts with an f</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>West Side Story</t>
+          <t>faggot</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>in kohlberg's theory of moral development which is the highest stage</t>
+          <t>poems that use the first letter of a word</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Stage six (universal ethical principles driven)</t>
+          <t>acrostic</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>who is the presiding officer in the house</t>
+          <t>who is the most decorated winter olympian in history</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>The Speaker of the House</t>
+          <t>Norwegian cross-country skier Marit Bjørgen</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>who dies in grey's anatomy season 8 plane crash</t>
+          <t>who is the author of the book of luke in the bible</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Dr. Lexie Grey</t>
+          <t>Luke the companion of Paul</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>who played the abominable snowman in monsters inc</t>
+          <t>what fraction of the british population was killed by the black death</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>John Dezso Ratzenberger</t>
+          <t>40–60%</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>who is the mother of moses in the holy bible</t>
+          <t>who is the speaker of the house in the house of representatives</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Jochebed</t>
+          <t>Congressman Paul Ryan from Wisconsin</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>when did never gonna give you up come out</t>
+          <t>what is the meaning of divergent in the movie</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>27 July 1987</t>
+          <t>equal attributes of multiple factions</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>world's first steamship driven by a screw propeller</t>
+          <t>who is the actor that plays wonder woman</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>SS Archimedes</t>
+          <t>Gal Gadot</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>pet shop boys' first uk number one single</t>
+          <t>who wrote the score to lord of the rings</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>"West End Girls"</t>
+          <t>Howard Leslie Shore</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>which actress helped create the voice of et</t>
+          <t>where is the invictus games being held 2017</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Pat WelshDebra Winger</t>
+          <t>Toronto, Ontario, Canada</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>zend avesta is the holy book of which religion</t>
+          <t>who plays ray palmer in dc legends of tomorrow</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Zoroastrianism</t>
+          <t>Brandon James Routh</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>what is an uruk hai in lord of the rings</t>
+          <t>ascites is one of the late features of</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>an advanced breed of orcs that serve Sauron and Saruman</t>
+          <t>liver cirrhosis</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>when did papua new guinea become an independent country</t>
+          <t>who sings with the rolling stones gimme shelter</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>16 September 1975</t>
+          <t>Merry Clayton</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>who died on grey's anatomy plane crash</t>
+          <t>shift from one key to another within a composition</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Dr. Lexie Grey</t>
+          <t>modulation</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>who's the killer in i still know</t>
+          <t>how many goals messi scored in world cup 2006</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2948,7 +2948,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Ben</t>
+          <t>once in 2006</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>who sang it must have been love in pretty woman</t>
+          <t>where was the opening scene of the sound of music filmed</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Roxette</t>
+          <t>at Mehlweg mountain near the town of Marktschellenberg in Bavaria</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>which province of canada has a large french population</t>
+          <t>when did the first superman movie come out</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Quebec</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>who sings the song you find out who your friends are</t>
+          <t>how big is a sheet of printer paper</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Tracy Lawrence</t>
+          <t>8.5 by 11.0 inches (215.9 by 279.4 mm)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>who plays cindy lou who in the grinch that stole christmas</t>
+          <t>when were the books of the hebrew bible written</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Taylor Michel Momsen</t>
+          <t>the 5th century BCE</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>when was the term political correctness first used</t>
+          <t>where was kenny chesney anything but mine filmed</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>Malibu, California and Myrtle Beach, South Carolina</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>who is next in line for the british thrown</t>
+          <t>what is coreldraw for what purpose we use this software</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Charles, Prince of Wales</t>
+          <t>a vector graphics editor developed and marketed by Corel Corporationto edit two-dimensional images such as logos and posters</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>who set the fires in little fires everywhere</t>
+          <t>when was texas annexed to the united states</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Izzy</t>
+          <t>December 29, 1845</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3240,7 +3240,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>when does wilson find out he has cancer</t>
+          <t>who was in charge of building the eiffel tower</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Season 8 episode "Body and Soul"</t>
+          <t>Alexandre Gustave Eiffel (born Bönickhausen</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>where does the running of the bulls end</t>
+          <t>what is the ribbon colour of vir chakra</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>the bullring</t>
+          <t>half dark blue and half orange-saffron</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>who was the explorer that reached the cape of good hope at the southern tip of africa</t>
+          <t>who wrote the first testament of the bible</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3338,7 +3338,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Bartolomeu Dias</t>
+          <t>Israelites</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>who played seven of nine on star trek</t>
+          <t>when was the european research laboratory (columbus) launched</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Jeri Lynn Ryan</t>
+          <t>February 7, 2008</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>what was king kong's fur made out of</t>
+          <t>who did massachusetts send to london to negotiate the legality of their charter</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3416,7 +3416,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>bearskin</t>
+          <t>Increase Mather</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>who dies in the plane crash grey's anatomy season 8</t>
+          <t>where are most peanuts grown in the us</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Dr. Lexie Grey (Chyler Leigh)</t>
+          <t>the southeastern United States region which includes Alabama, Georgia, and Floridathe southwestern United States region which includes New Mexico, Oklahoma, and Texasthe general eastern United States which include Virginia, North Carolina, and South Carolina</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>what is the first book in the magnus chase series</t>
+          <t>who killed robert baratheon in game of thrones</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>The Sword of Summer</t>
+          <t>Cersei</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>who's picture is on the $50 bill</t>
+          <t>who plays the voice of steve on american dad</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Ulysses S. Grant</t>
+          <t>Steve Smith</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>when did the uk get rid of capital punishment</t>
+          <t>who sang the original song the sound of silence</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>Simon &amp; Garfunkel</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3591,7 +3591,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>the pangolakha wildlife sanctuary (pws) is located in which state</t>
+          <t>where does the smell of the skunk go</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Sikkim</t>
+          <t>anal scent glands</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>how and when was knowledge of paper making established in christian europe</t>
+          <t>when does the playclock start in the nfl</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>1282</t>
+          <t>the end of the previous down</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>who said these are times that try men's souls</t>
+          <t>the super cyclone which slammed orissa in 1999 was with an approximate wind speed of</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Paine</t>
+          <t>260 km/h (160 mph)</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>who gave the presidential address in the resolution of lahore</t>
+          <t>who is responsible for starting the nordic games and presenting the idea for the winter olympics</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Sir Shah Nawaz Khan of Mamdot</t>
+          <t>Viktor Balck</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>actress who played alice on the brady bunch</t>
+          <t>when did the anaheim angels change their name</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Ann Bradford Davis</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>who has ian beale been married to in eastenders</t>
+          <t>where is it written in the bible jesus wept</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Cindy WilliamsMel HealyLaura Dunntwice to Jane Collins</t>
+          <t>Gospel of John, chapter 11, verse 35</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>when did soul train go off the air</t>
+          <t>what does an abscess look like on skin</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>March 25, 2006</t>
+          <t>rednessswelling</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>measurement system whose divisions are powers of ten</t>
+          <t>who plays bernard the elf in santa clause</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>the metric system</t>
+          <t>David Krumholtz</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>where is the invictus games being held 2017</t>
+          <t>what was the first british colony in america</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Toronto, Ontario, Canada</t>
+          <t>1607 in Jamestown, Virginia</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -3942,7 +3942,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>when did the letter j become apart of the alphabet</t>
+          <t>when did the first printing press come out</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>and</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>who sang the original shake your tail feather</t>
+          <t>how many chapters are there in the book of esther</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>The Five Du-Tones</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>who wrote the majority opinion in mcdonald v. chicago</t>
+          <t>who got stabbed in lord of the flies</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Justice AlitoJustice Thomas</t>
+          <t>Captain Benson</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>where is the bar in it's always sunny in philadelphia</t>
+          <t>who does muriel marry in muriel's wedding</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>South Philadelphia</t>
+          <t>South African swimmer David Van Arkle</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>who sang the original song the sound of silence</t>
+          <t>what is the currency of papua new guinea</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Simon &amp; Garfunkel</t>
+          <t>kina</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4137,7 +4137,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>where was malaysia flight 370 supposed to land</t>
+          <t>when is the new season of young sheldon coming out</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4157,7 +4157,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Beijing Capital International Airport</t>
+          <t>September 24, 2018</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>is the three little pigs a fairy tale or folktale</t>
+          <t>what is the term for a female reproductive cell apex</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>folktale</t>
+          <t>the ovule</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>what is the first book in the skulduggery pleasant series</t>
+          <t>where was 20 million miles to earth filmed</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Skulduggery Pleasant</t>
+          <t>Rome, Italythe U.S.</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>when does daylight savings time end in colorado</t>
+          <t>when have man city won the premier league</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>first Sunday in November</t>
+          <t>2012 and 2014</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -4293,7 +4293,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>which part of the digestive tract runs through the diaphragm</t>
+          <t>where does the lily of the valley grow</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>thoracic diaphragm</t>
+          <t>throughout the cool temperate Northern Hemisphere in Asia, and Europe</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>who played gibbs in pirates of the caribbean</t>
+          <t>when did the brown vs board of education end</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Kevin Robert McNally</t>
+          <t>May 17, 1954</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>what is the system of measurement used in the us</t>
+          <t>what is the status of the dream act</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>United States customary units</t>
+          <t>has failed to pass</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>what is the american league record for most consecutive wins</t>
+          <t>why is hershel keeping walkers in the barn</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2017 Cleveland Indians at 22</t>
+          <t>Hershel believes they are still peopleand can be cured</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>when did spike island close as a prison</t>
+          <t>what is an example of an internal stimulus</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4469,7 +4469,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>Homeostatic imbalances</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>girl who plays piper in orange is the new black</t>
+          <t>who played clara on the andy griffith show</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Taylor Schilling</t>
+          <t>Sarah Hope Summers</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>when is a free throw awarded in basketball</t>
+          <t>who says the opening of law and order svu</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>after a foul on the shooter by the opposing team</t>
+          <t>Steven M. Zirnkilton</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>how many all india services are there in india</t>
+          <t>where is an eye for an eye found in the bible</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>three</t>
+          <t>ExodusLeviticusDeuteronomy</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>materials that clearly transmit visible light are said to be</t>
+          <t>who played snow queen in once upon a time</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>optically transparent</t>
+          <t>Elizabeth Mitchell</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>who won the oscar for best actor in 2014</t>
+          <t>when was the last time a wolverine was seen in michigan</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Matthew McConaughey</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>how much did disney buy star wars franchise for</t>
+          <t>first new zealander to run a mile in under four minutes</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>$4.06 billion</t>
+          <t>John Walker</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>where is the biggest guinness brewery in the world</t>
+          <t>when was the last time someone got swept in the nba finals</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>when was human league don't you want me released</t>
+          <t>who is the writer on once upon a time</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>27 November 1981</t>
+          <t>Edward KitsisEdward Kitsis</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -4800,7 +4800,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>what nfl team does jj watt's brother play for</t>
+          <t>where is area code 616 in united states</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Los Angeles ChargersPittsburgh Steelers</t>
+          <t>the west-central portion of the Lower Peninsula of Michigan</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>what is the setting of rip van winkle by washington irving</t>
+          <t>who plays bonnie's voice on family guy</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>In a pleasant village, at the foot of New York's Catskill Mountains</t>
+          <t>Jennifer Tilly</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>who sang the original i love rock and roll</t>
+          <t>what is make it stop by rise against about</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>the Arrows</t>
+          <t>It Gets Better campaign</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>when did the first smart cell phone come out</t>
+          <t>who is the guru of karan in mahabharat</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -4937,7 +4937,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>Parashurama</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>what is the most dangerous snake in the united states</t>
+          <t>what is the official flower of the belmont stakes</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>eastern and western diamondback rattlesnake</t>
+          <t>white carnations</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>what came first mean machine or the longest yard</t>
+          <t>what is made up of charged particles that continually escape from the corona</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -5015,7 +5015,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>The Longest Yard</t>
+          <t>solar wind</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>the conversion of a thiol into a disulfide occurs by what type of chemical reaction</t>
+          <t>who tried to steal the declaration of independence</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>coupling of two thiol groups</t>
+          <t>Benjamin Franklin Gates</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>how many cross lanes are there in kho kho</t>
+          <t>who plays the science officer in star trek discovery</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>eight</t>
+          <t>Anthony Rapp</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>who is required to file a flight plan</t>
+          <t>a measure using algorithms to publically protect patient identifiable information is</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5132,7 +5132,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>pilotflight dispatcher</t>
+          <t>k-anonymization</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>when was the last time the cavs won a championship</t>
+          <t>who sings gentle on my mind at the end of i'll be me</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>The Band Perry</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>when was the curious incident of the dog in the nighttime published</t>
+          <t>who is carries parents on days of our lives</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2003</t>
+          <t>Anna DiMeraRoman Brady</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>where in the uk were the anchors and chains for the rms titanic made</t>
+          <t>when did the first smart cell phone come out</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Netherton</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -5268,7 +5268,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>factors that led to the rise of monarchy in israel</t>
+          <t>what part of the computer hardware only retains data while the computer is on</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5288,7 +5288,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>large popular expression in favour of introducing a king</t>
+          <t>random-access memory (RAM)</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>who wrote the song i would rather go blind</t>
+          <t>who plays chekov in the new star trek</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -5327,7 +5327,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Ellington Jordan</t>
+          <t>Anton Viktorovich Yelchin</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>how long does it take for a maine coon cat to be fully grown</t>
+          <t>when does lady and the tramp take place</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>three to five years</t>
+          <t>in a quaint Midwestern town</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>who played gabriel in the original far from the madding crowd</t>
+          <t>town meetings practiced in many small new england towns are examples of what</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -5405,7 +5405,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Alan Bates</t>
+          <t>direct democratic rule</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>when will the new predator movie be released</t>
+          <t>what's the name of he man's cat</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5444,7 +5444,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>September 14, 2018</t>
+          <t>Battle Cat</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -5463,7 +5463,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>what is the meaning of radius of gyration</t>
+          <t>average number of trophic level in the food chain of an ecosystem are</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>the radial distance of a point from the axis of rotation at which, if whole mass of the body is assumed to be concentrated, its moment of inertia about the given axis would be the same as with its actual distribution of mass</t>
+          <t>5 or 6</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>where is i am that i am in the bible</t>
+          <t>where is the external oblique located in the body</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Exodus 3:14</t>
+          <t>on the lateral and anterior parts of the abdomen</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>who used viruses to determine that dna was the molecule of heredity</t>
+          <t>who discovered the fact that south america was a separate continent</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Alfred HersheyMartha Chase</t>
+          <t>Amerigo VespucciGonçalo Coelho</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -5580,7 +5580,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>where is the next world fair to be held</t>
+          <t>who played lois lane in superman the movie</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>"Margot" Kidder</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>who played michael corleone italian wife in the godfather</t>
+          <t>where is the kola peninsula located on a map</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -5639,7 +5639,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Simonetta Stefanelli</t>
+          <t>in the far northwest of Russiainside the Arctic Circle</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>where does lily of the valley come from</t>
+          <t>who wrote the musical score for the godfather</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>native throughout the cool temperate Northern Hemisphere in Asia, and Europe</t>
+          <t>Giovanni "Nino" Rota</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>when was texas added to the united states</t>
+          <t>who plays general iroh in avatar the last airbender</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>December 29, 1845</t>
+          <t>Mako IwamatsuGreg Baldwin</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>where is the external oblique located in the body</t>
+          <t>what was the name of columbo's dog</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -5756,7 +5756,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>on the lateral and anterior parts of the abdomen</t>
+          <t>"Dog"</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>who shot ej dimera on days of our lives</t>
+          <t>what was the war guilt clause in the treaty of versailles</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>his disloyal bodyguard, Miguel</t>
+          <t>the opening article of the reparations section of the Treaty of Versailles, which ended the First World War between the German Empire and the Allied and Associated Powers</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>where do the tannins in wine come from</t>
+          <t>who wrote the book upon which the last picture show was based</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -5834,7 +5834,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>plant pigmentsphenolic compounds</t>
+          <t>Larry McMurtry</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -5853,7 +5853,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>who played the holographic doctor on star trek</t>
+          <t>what did the european export from the caribbean</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Robert Picardo</t>
+          <t>sugarrummolasses</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>when did lane splitting become legal in california</t>
+          <t>who was known as the mother of the iditarod</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>August, 2016</t>
+          <t>Dorothy G. Page</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>what is the main source of heat and light energy</t>
+          <t>who sings the immigrant song in the girl with the dragon tattoo</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Incandescence</t>
+          <t>Karen O</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -5970,7 +5970,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>who is the youngest us president elected to the office</t>
+          <t>in january of 1973 a ceasefire in vietnam was signed by all of the following except</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>John F. Kennedy</t>
+          <t>United States Senate</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>who plays the voice of steve on american dad</t>
+          <t>when did us give up control of panama canal</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -6029,7 +6029,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Steve Smith</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -6048,7 +6048,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>where was the movie safe haven filmed at</t>
+          <t>in javanese gamelan music typical elaborating instruments are</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6068,7 +6068,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>WilmingtonSouthport, North CarolinaLouisianaon the Linn Cove Viaduct along the Blue Ridge Parkway near Grandfather Mountain in Linville, North Carolina</t>
+          <t>percussive</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>when did imagine dragons first song come out</t>
+          <t>a million ways to die in the west filming locations</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>Albuquerque, New MexicoSanta Fe Studio in Santa Fe</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>when does new season of tokyo ghoul start</t>
+          <t>where does the movie what if take place</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>Toronto, Ontario</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>what is an example of an internal stimulus</t>
+          <t>distribution of power between centre and state in indian constitution is based on which scheme</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -6185,7 +6185,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Homeostatic imbalances</t>
+          <t>a federal structure</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>what iq do you need to be in mensa</t>
+          <t>what is the bengali name of peepal tree</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>132148</t>
+          <t>ashwattha tree</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>what was the supreme court ruling on plessy versus ferguson</t>
+          <t>where does call of duty ww2 take place</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -6263,7 +6263,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>upheld the constitutionality of racial segregation laws for public facilities as long as the segregated facilities were equal in quality, a doctrine that came to be known as "separate but equal"</t>
+          <t>in European theatre of the war</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>where does most of the oil in the us come from</t>
+          <t>what is it called when you blur the background in a photo</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>the U.S.</t>
+          <t>, bokeh</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -6321,7 +6321,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>what grade is matt saracen in in season 1</t>
+          <t>when does singin in the rain take place</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>sophomore</t>
+          <t>the late 1920s</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -6360,7 +6360,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>poem on the pedestal of the statue of liberty</t>
+          <t>when did they stop making pennies in canada</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -6380,7 +6380,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>"The New Colossus"</t>
+          <t>May 2012</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -6399,7 +6399,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>when did womens hockey start in the olympics</t>
+          <t>when was first constituent assembly held in nepal</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>May 28, 2008</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -6438,7 +6438,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>where was tomorrow where the war began filmed</t>
+          <t>what is a homogeneous mixture in physical science</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>the Hunter Region of New South Wales, AustraliaHunterRaymond TerraceHistoric King StreetMaitlandthe Blue Mountainsthe Luskintyre bridgeThe Fox Studios site in SydneyTerrey Hills in northern Sydney</t>
+          <t>a solid, liquid or gaseous mixture that has the same proportions of its components throughout a given sample</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -6477,7 +6477,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>first nhl player to score a hat trick</t>
+          <t>when did stink bugs come to the us</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Harry Hyland</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -6516,7 +6516,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>who sang what we need is a great big melting pot</t>
+          <t>who sings lips of an angel country version</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Blue Mink</t>
+          <t>Jack Ingram</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -6555,7 +6555,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>what is tom's full name in to kill a mockingbird</t>
+          <t>who was edwards dating on grey's anatomy</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -6575,7 +6575,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Tom Robinson</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>what is the proximal attachment of the flexor carpi ulnaris in humans</t>
+          <t>the type of reproduction that requires the union of sperm and egg</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>humeralulnar</t>
+          <t>Human fertilization</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>when did gods not dead 3 come out</t>
+          <t>iron pillar near qutub minar built by whom</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -6653,7 +6653,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>March 30, 2018</t>
+          <t>king Chandra</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>when did the new orleans saints win the superbowl</t>
+          <t>when is a defendant entitled to have bail returned</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -6692,7 +6692,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>February 7, 2010</t>
+          <t>may be returned at the end of the trial, if all court appearances are made, regardless of whether the person is found guilty or not guilty of the crime accused.</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>what is airplane mode on an android phone</t>
+          <t>who is the song she'll be coming round the mountain about</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>a setting available on smartphones and other portable computers that, when activated, suspends radio-frequency signal transmission by the device, thereby disabling Bluetooth, telephony, and Wi-Fi</t>
+          <t>the Second Coming of Christ and subsequent Rapture</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -6750,7 +6750,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>how big is a sheet of printer paper</t>
+          <t>what type of motor is used in most electric power steering (eps) systems</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>8.5 by 11.0 inches (215.9 by 279.4 mm)</t>
+          <t>electric motors</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -6789,7 +6789,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>what year was the great fire of rome</t>
+          <t>who wrote the song you're welcome from moana</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -6809,7 +6809,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>AD 64</t>
+          <t>Lin-Manuel MirandaMark MancinaOpetaia Foa'i</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>when did the anaheim angels change their name</t>
+          <t>what is the first book in the skulduggery pleasant series</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>Skulduggery Pleasant</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>who devised the technique syllogism to learn logic</t>
+          <t>when did texas gain independence and become a republic</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -6887,7 +6887,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Aristotle</t>
+          <t>March 2, 1836</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>when did john snow come back to life</t>
+          <t>when was the last time the patriots went to the superbowl</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>The Red Woman</t>
+          <t>2016–17</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -6945,7 +6945,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>where did the names of the week come from</t>
+          <t>who did david ryall play in call the midwife</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -6965,7 +6965,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>names of the classical planets in Hellenistic astrology, which were in turn named after contemporary deities, a system introduced in by the Roman Empire during Late Antiquity</t>
+          <t>Tommy Mills</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -6984,7 +6984,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>where did industrialization first took place in the united states</t>
+          <t>who is the owner of the washington post</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Rhode Island</t>
+          <t>Nash Holdings</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -7023,7 +7023,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>what kind of ruler has absolute authority over his subjects</t>
+          <t>how many died in the las vegas shooting</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -7043,7 +7043,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Absolute monarchy, or despotic monarchy</t>
+          <t>58</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -7062,7 +7062,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>who wrote the music and lyrics for my fair lady</t>
+          <t>when did the federal student loan program start</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -7082,7 +7082,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>lyrics by Alan Jay Lernermusic by Frederick Loewe</t>
+          <t>1960s</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -7101,7 +7101,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>who wrote the song living on a prayer</t>
+          <t>who sings the song dude looks like a lady</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -7121,7 +7121,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Jon Bon JoviRichie SamboraDesmond Child</t>
+          <t>Aerosmith</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>who was the pilot of the plane that dropped the bomb on nagasaki</t>
+          <t>what is the role of a navy frigate</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Major General Charles W. Sweeney</t>
+          <t>used to protect other warships and merchant-marine ships, especially as anti-submarine warfare (ASW) combatants for amphibious expeditionary forces, underway replenishment groups, and merchant convoys</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>where are most of the divergent boundaries found</t>
+          <t>who used viruses to determine that dna was the molecule of heredity</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>between oceanic plates</t>
+          <t>Alfred HersheyMartha Chase</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>when did the british parliament pass the indian independence bill</t>
+          <t>the manubrium body and xiphoid process are portions of the</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>18 July 1947</t>
+          <t>sternum</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>who was the girl who was blind and deaf</t>
+          <t>who wrote willy wonka and the chocolate factory</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -7277,7 +7277,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Helen Adams Keller</t>
+          <t>Roald DahlDavid Seltzer</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>where would the oldest oceanic crust be found</t>
+          <t>where was the movie true grit filmed with john wayne</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -7316,7 +7316,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>away from the ridges</t>
+          <t>Ouray County, Colorado</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>who does aslan represent in the lion the witch and the wardrobe</t>
+          <t>what did the chinese use oracle bones for</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -7355,7 +7355,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Jesus Christ</t>
+          <t>pyromancy</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>sons of anarchy what is wrong with clay's hands</t>
+          <t>what hotel was the las vegas shooting in</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>suffers from osteoarthritis (degenerative arthritis) in his hands, which is slowly worsening</t>
+          <t>Mandalay Bay hotel</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -7413,7 +7413,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>what are tiny pores present on the surface of leaf called</t>
+          <t>what are the coordinates for the south pole of the moon</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -7433,7 +7433,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>stomates</t>
+          <t>80°S to 90°S</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -7452,7 +7452,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>theater is classified as which type of art</t>
+          <t>who won the wwe elimination chamber in 2018</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -7472,7 +7472,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>performing</t>
+          <t>Roman Reigns</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>when did anchor butter stop being from new zealand</t>
+          <t>amendment giving the us the right of intervention in panama</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>August 2012</t>
+          <t>The 1904 constitution</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -7530,7 +7530,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>who won the mens singles at wimbledon this year</t>
+          <t>what rank is lieutenant colonel in the army</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Novak Djokovic</t>
+          <t>a field grade military officer rank just above the rank of major and just below the rank of colonel</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -7569,7 +7569,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>where does the small intestine join the large intestine</t>
+          <t>in computers which is still used for doing payroll and accounting</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -7589,7 +7589,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>the ileocecal valve</t>
+          <t>Payroll automation</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>who owns the pioneer casino in laughlin nv</t>
+          <t>who gets to be the speaker of the house</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -7628,7 +7628,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Archon Corporation</t>
+          <t>presiding officer of the United States House of Representatives</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>who is the author of the man booker prize winning book life of pi</t>
+          <t>what did the u.s. policy called the truman doctrine promise to do</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -7667,7 +7667,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Yann Martel</t>
+          <t>created to counter Soviet geopolitical expansion during the Cold War</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>where is the shutter speed located on a camera</t>
+          <t>what category was ivan when it hit florida</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -7706,7 +7706,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>digital sensor inside the camera</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>what type of motor is used in most electric power steering (eps) systems</t>
+          <t>who wrote manfred mann's blinded by the light</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -7745,7 +7745,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>electric motors</t>
+          <t>Bruce Springsteen</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>who plays the black panther in captain america</t>
+          <t>in the late-nineteenth century the european race to rapidly colonize africa became known as the</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -7784,7 +7784,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Chadwick Aaron Boseman</t>
+          <t>Scramble for Africa</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -7803,7 +7803,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>when did the mudslide happen in sierra leone</t>
+          <t>when was the last time houston rockets made the finals</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>August 14, 2017</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>a bundle of sticks that starts with an f</t>
+          <t>what finger do u put a wedding ring on</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>faggot</t>
+          <t>finger between the middle finger and the little finger</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>where does water enter the vascular system of a starfish</t>
+          <t>where is mount sinai located in the bible</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>madreporite</t>
+          <t>Book of Exodusother books</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>when does the school year start in israel</t>
+          <t>where does the cadenza usually occur in a concerto</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>September 1</t>
+          <t>near the end of the first movement</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>who makes laws for the state in india</t>
+          <t>the great majority of which tracts pass through the corpus callosum</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -7979,7 +7979,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>the State Governments</t>
+          <t>commissural fibers</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
@@ -7998,7 +7998,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>who plays grace's boyfriend in frankie and grace</t>
+          <t>i can see clearly now the rain has gone original singer</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -8018,7 +8018,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Sam Elliott</t>
+          <t>Johnny Nash</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
@@ -8037,7 +8037,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>when did the us begin using daylight savings time</t>
+          <t>when did mount st helens blew its top off</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -8057,7 +8057,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>1918</t>
+          <t>8:32:17 a.m. PDT (UTC−7) on Sunday, May 18, 1980</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
@@ -8076,7 +8076,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>the most expensive roller coasters in the world</t>
+          <t>what did cro-magnon man paint on cave walls</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -8096,7 +8096,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Expedition Everest — Legend of the Forbidden Mountain</t>
+          <t>animals</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>the river separates india as north and south</t>
+          <t>where is the women's world cup being held</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -8135,7 +8135,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Narmada RiverMahanadi river</t>
+          <t>England</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -8154,7 +8154,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>first indian man to win olympic gold medal</t>
+          <t>which is the characteristic of a line width depth color length</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -8174,7 +8174,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Abhinav Bindra</t>
+          <t>widthlength</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -8193,7 +8193,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>who is the most decorated winter olympian in history</t>
+          <t>a permanent magnet is a magnet made from a material that</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -8213,7 +8213,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Norwegian cross-country skier Marit Bjørgen</t>
+          <t>is magnetized and creates its own persistent magnetic field</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
@@ -8232,7 +8232,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>who determines the offer price in a dutch auction</t>
+          <t>what is the cathedral of art in mexico</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -8252,7 +8252,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>the auctioneer</t>
+          <t>Palacio de Bellas Artes</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -8271,7 +8271,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>what's the name of the new tomb raider movie</t>
+          <t>how much horsepower does a 2005 chrysler 300c have</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Tomb Raider</t>
+          <t>340</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -8310,7 +8310,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>if you are from dubai what are you called</t>
+          <t>who invented the first printing press in 1450</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -8330,7 +8330,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Emirati</t>
+          <t>Johannes Gutenberg</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
@@ -8349,7 +8349,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>what do you call that type of asexual reproduction yeast</t>
+          <t>what is the main religion of the dominican republic</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -8369,7 +8369,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>budding</t>
+          <t>Catholicism</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -8388,7 +8388,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>how many general partners in a limited partnership</t>
+          <t>from which body part shurpnakha drive her name</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>at least one</t>
+          <t>fingernails</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
@@ -8427,7 +8427,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>where is most of the chlorophyll in a plant located</t>
+          <t>when does the new southpark season come out</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -8447,7 +8447,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>cyanobacteriachloroplasts</t>
+          <t>September 13, 2017</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>what is in the center of the milky way galaxy</t>
+          <t>how many teams havent won the stanley cup</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -8486,7 +8486,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>a supermassive black hole</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -8505,7 +8505,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>who plays bernard the elf in santa clause</t>
+          <t>who led a gang of outlaws in sherwood forest</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>David Krumholtz</t>
+          <t>Robin</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>all the light we cannot see french town</t>
+          <t>what was the purpose of the second great awakening</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Saint-Malo</t>
+          <t>reflected Romanticismrejected the skeptical rationalism and deism</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>which character from greek mythology can be described as being strong</t>
+          <t>how far is las vegas from mesquite nevada</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -8603,7 +8603,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>Heracles</t>
+          <t>80 miles</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
@@ -8622,7 +8622,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>who plays dr shepherd on grey's anatomy</t>
+          <t>when does ralph break the internet come out</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -8642,7 +8642,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Patrick Dempsey</t>
+          <t>November 21, 2018</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -8661,7 +8661,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>when was joseph and the technicolor dreamcoat written</t>
+          <t>when did mario kart come out on wii</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -8681,7 +8681,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>April 2008</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -8700,7 +8700,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>after how much time we can withdraw money from ppf</t>
+          <t>who has won the boat race more times</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>from the start of the seventh financial year.</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -8739,7 +8739,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>who played mike tv in willy wonka 2005</t>
+          <t>who played the father on what's happening</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Paris Themmen</t>
+          <t>Thalmus Rasulala</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
@@ -8778,7 +8778,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>who wrote to kill a mockingbird and in what year was it published</t>
+          <t>who has been appointed chief justice of india</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -8798,7 +8798,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Nelle Harper Lee1960</t>
+          <t>Dipak Misra</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
@@ -8817,7 +8817,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>who has the right of way in international waters</t>
+          <t>where are voltage gated sodium channels concentrated in myelinated axons</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -8837,7 +8837,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Neither vessel</t>
+          <t>plasma membrane</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
@@ -8856,7 +8856,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>who sings just shut up and dance with me</t>
+          <t>what part of the constitution talks about the electoral college</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -8876,7 +8876,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Walk the Moon</t>
+          <t>Twelfth Amendment</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>when did america switch from tea to coffee</t>
+          <t>who do you play as in life is strange before the storm</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>1773</t>
+          <t>sixteen-year-old Chloe Price</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>how far is las vegas from mesquite nevada</t>
+          <t>the national science day is observed every year on 28 february in honour of</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>80 miles</t>
+          <t>Sir Chandrashekhara Venkata Raman</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -8973,7 +8973,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>who won the ladies figure skating in sochi</t>
+          <t>when was the old beauty and the beast released</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>Adelina Sotnikova</t>
+          <t>19911946</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>what is the shortest player in the nfl</t>
+          <t>who defended the soldiers involved in the boston massacre during their trial</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -9032,7 +9032,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Trindon Jerard Holliday</t>
+          <t>John Adams</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>how old do you need to be to serve alcohol in wisconsin</t>
+          <t>where did steph curry play college basketball at</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>Davidson College</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -9090,7 +9090,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>who came up with the teenage mutant ninja turtles</t>
+          <t>dead poets society what play is neil in</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -9110,7 +9110,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>Kevin EastmanPeter Laird</t>
+          <t>A Midsummer Night's Dream</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>who said houston we have a problem in the movie apollo 13</t>
+          <t>who was the oldest elected president of the united states of america</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -9149,7 +9149,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>actor Tom Hanks, portraying Mission Commander Jim Lovell</t>
+          <t>Donald Trump</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>what are the names of the 5 villages in cinque terre</t>
+          <t>lok sabha or rajya sabha which is bigger</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -9188,7 +9188,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Monterosso al MareVernazzaCornigliaManarolaRiomaggiore</t>
+          <t>Lok Sabha</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>when was the last time the patriots went to the superbowl</t>
+          <t>when did the new england patriots change their logo</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>2016–17</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -9246,7 +9246,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>last president to get lifetime secret service protection</t>
+          <t>while writing time the number after the two dots stands for</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -9266,7 +9266,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Barack Obama</t>
+          <t>minutes</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -9285,7 +9285,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>who plays alan in last tango in halifax</t>
+          <t>who sings a nice day for a white wedding</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -9305,7 +9305,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Sir Derek Jacobi</t>
+          <t>Billy Idol</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -9324,7 +9324,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>what episode of adventure time is marshall lee in</t>
+          <t>who sings you just call out my name</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -9344,7 +9344,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>Bad Little Boy</t>
+          <t>The Weeknd</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>what engines do they use in formula 1</t>
+          <t>who illustrated the original winnie the pooh books</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -9383,7 +9383,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>1.6 litre V6 turbo engines</t>
+          <t>E. H. Shepard</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>who illustrated the original winnie the pooh books</t>
+          <t>where did the term space cadet come from</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -9422,7 +9422,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>E. H. Shepard</t>
+          <t>a 1948 science fiction novel by Robert A. Heinlein</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -9441,7 +9441,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>what kind of habitat do river otters live in</t>
+          <t>what type of poem is love among the ruins</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -9461,7 +9461,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>a burrow close to the water's edge in river, lake, swamp, coastal shoreline, tidal flat, or estuary ecosystems</t>
+          <t>rhyming couplets in which long trochaic lines are paired with short lines of three syllables</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -9480,7 +9480,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>who plays john in last tango in halifax</t>
+          <t>when did scotland abolish the authority of the pope</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -9500,7 +9500,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Tony Gardner</t>
+          <t>August 1560</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -9519,7 +9519,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>where is the world tallest building the burj khalifa located</t>
+          <t>who plays charlie on it's always sunny in philadelphia</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>Charles Peckham Day</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>who wrote the music for twinkle twinkle little star</t>
+          <t>how many cubes are in a 5x5x5 cube</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Jane Taylor</t>
+          <t>98</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>what category was ivan when it hit florida</t>
+          <t>where is the baseball all-star game being played</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -9617,7 +9617,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>July 11, 2017</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -9636,7 +9636,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>which soil is found suitable for growing coffee in india</t>
+          <t>how many cross lanes are there in kho kho</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -9656,7 +9656,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>well drained soil conditions</t>
+          <t>eight</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -9675,7 +9675,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>who sang the opening theme song for wkrp in cincinnati</t>
+          <t>in 2016 who became the ceo of wipro company</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Steve Carlisle</t>
+          <t>Abid Ali Neemuchwala</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>how many times has widespread panic played red rocks</t>
+          <t>who is the dancer on thinking out loud</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>Brittany Cherry</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>when was the first gas field discovered in bangladesh</t>
+          <t>when was the first car made in united states</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -9773,7 +9773,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>1955</t>
+          <t>1890s</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -9792,7 +9792,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>which country had taken lead in establishing saarc</t>
+          <t>where would the oldest oceanic crust be found</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -9812,7 +9812,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>away from the ridges</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -9831,7 +9831,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>when was the last year lead paint was used</t>
+          <t>what are the in the night garden characters</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -9851,7 +9851,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>Iggle PiggleMakka PakkaUpsy Daisythe Tombliboosthe Pontipines / the Wottingersthe Haahoosthe Ninky Nonkthe Pinky Ponk</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -9870,7 +9870,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>who played winston churchhill in the darkest hour</t>
+          <t>who was the maratha peshwa when the third battle of panipat was fought</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>Gary Oldman</t>
+          <t>Madhavrao</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -9909,7 +9909,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>where is the yucatan peninsula located in mexico</t>
+          <t>when was the first vampire diaries episode released</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -9929,7 +9929,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>in southeastern Mexico, separates the Caribbean Sea from the Gulf of Mexico, with the northern coastline on the Yucatán Channel</t>
+          <t>September 10, 2009</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -9948,7 +9948,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>in the arms of an angel song in movie</t>
+          <t>who is the youngest us president elected to the office</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -9968,7 +9968,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>A Dog Named Christmas</t>
+          <t>John F. Kennedy</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -9987,7 +9987,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>where are the digestive enzymes found in a cell</t>
+          <t>who made heard it through the grapevine first</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -10007,7 +10007,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>in their lysosomes</t>
+          <t>Gladys Knight &amp; the Pips</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>when do new stranger things episodes come out</t>
+          <t>when does the 2018 regular baseball season start</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -10046,7 +10046,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>late 2018 or early 2019</t>
+          <t>March 29, 2018</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -10065,7 +10065,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>what are the main functions of the control bus</t>
+          <t>the initial structure for british bomb disposal parties in 1939 was composed of</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -10085,7 +10085,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>communicating with other devices within the computercarries commands from the CPUreturns status signals from the devices</t>
+          <t>ten sections, each section having a bomb disposal officer and 14 other ranks to assist</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>how many cards in hand magic the gathering</t>
+          <t>what is the name of the car in tarzan movie</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -10124,7 +10124,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>seven</t>
+          <t>Tarzan</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>who was the commander of the allied forces in europe</t>
+          <t>where is great britain located on the world map</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -10163,7 +10163,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>U.S. General Curtis M. Scaparrotti</t>
+          <t>in the north Atlantic Ocean off the northwest coast of continental Europe</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>what type of microsoft server serves as an email server</t>
+          <t>which u.s. general was the architect of the berlin airlift</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Microsoft Exchange Server</t>
+          <t>Curtis Emerson LeMay</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">

</xml_diff>